<commit_message>
Add a "Summary" sheet to the articles xlsx
Simple stage-by-stage table (Stage | What we do | Main source of inspiration |
What we actually borrow | Links), matching an external table format. It
uses. Full detail table kept as a second sheet.
</commit_message>
<xml_diff>
--- a/docs/articles-by-pipeline-part.xlsx
+++ b/docs/articles-by-pipeline-part.xlsx
@@ -7,10 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Articles by pipeline part" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary (for Mariella)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full detail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Articles by pipeline part'!$A$1:$I$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary (for Mariella)'!$A$1:$E$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full detail'!$A$1:$I$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -485,6 +487,271 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>What we do</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Main source of inspiration</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>What we actually borrow</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Links</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Raw video + ordered transcript</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>DELTA</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Same weak supervision: no timestamps / boundaries / durations</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Mate &amp; Dimiccoli (internal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Semantic front-end</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Encode short video clips and transcript actions into a shared semantic space</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>OVTAS</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Frozen VLM visual/text similarity idea</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2602.21406</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Stage A: coarse alignment</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Build the cost and force actions to appear in transcript order</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>our existing monotonic DP + HiERO-StepG principle</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Strict monotonic ordered alignment</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2605.31227</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Stage B1: segment extent</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Find the confident temporal extent of each action around its coarse location</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>HiERO-StepG</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Query-conditioned boundary / segment expansion</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2605.31227</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Stage B2: exact transition</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Search specifically for the best crossover point</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>our formulation (+ CVA boundary-contrastive principle, MASRA LRCA)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Explicit GT-free semantic boundary localization</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/byeol3325/CVA_cvpr ; https://arxiv.org/abs/2605.03398</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Optional Stage C</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Improve frame / segment consistency if boundaries remain noisy</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>CLOT / D-CLOT</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Closed-loop segment / frame / prototype refinement</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://openaccess.thecvf.com/content/ICCV2025/papers/Bueno-Benito_CLOT_Closed_Loop_Optimal_Transport_for_Unsupervised_Action_Segmentation_ICCV_2025_paper.pdf ; https://arxiv.org/abs/2608.05877</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Optional Stage D</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Reason only about difficult boundaries</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>TOGA / VideoLLaMA3</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Expensive local VLM reasoning, selectively</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2506.09445 ; https://arxiv.org/abs/2501.13106</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Convert refined boundaries into dense Y*</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>DELTA</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Preserve the existing downstream interface</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Mate &amp; Dimiccoli (internal)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Add a "Summary (for Mariella)" sheet to the articles xlsx
Simple stage-by-stage table (Stage | What we do | Main source of inspiration |
What we actually borrow | Links), matching the format the co-intern's team
uses. Full detail table kept as a second sheet.
</commit_message>
<xml_diff>
--- a/docs/articles-by-pipeline-part.xlsx
+++ b/docs/articles-by-pipeline-part.xlsx
@@ -7,10 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Articles by pipeline part" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary (for Mariella)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full detail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Articles by pipeline part'!$A$1:$I$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary (for Mariella)'!$A$1:$E$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full detail'!$A$1:$I$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -485,6 +487,271 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>What we do</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Main source of inspiration</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>What we actually borrow</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Links</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Raw video + ordered transcript</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>DELTA</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Same weak supervision: no timestamps / boundaries / durations</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Mate &amp; Dimiccoli (internal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Semantic front-end</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Encode short video clips and transcript actions into a shared semantic space</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>OVTAS</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Frozen VLM visual/text similarity idea</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2602.21406</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Stage A: coarse alignment</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Build the cost and force actions to appear in transcript order</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>our existing monotonic DP + HiERO-StepG principle</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Strict monotonic ordered alignment</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2605.31227</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Stage B1: segment extent</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Find the confident temporal extent of each action around its coarse location</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>HiERO-StepG</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Query-conditioned boundary / segment expansion</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2605.31227</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Stage B2: exact transition</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Search specifically for the best crossover point</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>our formulation (+ CVA boundary-contrastive principle, MASRA LRCA)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Explicit GT-free semantic boundary localization</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/byeol3325/CVA_cvpr ; https://arxiv.org/abs/2605.03398</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Optional Stage C</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Improve frame / segment consistency if boundaries remain noisy</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>CLOT / D-CLOT</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Closed-loop segment / frame / prototype refinement</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://openaccess.thecvf.com/content/ICCV2025/papers/Bueno-Benito_CLOT_Closed_Loop_Optimal_Transport_for_Unsupervised_Action_Segmentation_ICCV_2025_paper.pdf ; https://arxiv.org/abs/2608.05877</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Optional Stage D</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Reason only about difficult boundaries</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>TOGA / VideoLLaMA3</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Expensive local VLM reasoning, selectively</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2506.09445 ; https://arxiv.org/abs/2501.13106</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Convert refined boundaries into dense Y*</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>DELTA</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Preserve the existing downstream interface</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Mate &amp; Dimiccoli (internal)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Actually apply the personal-name removal (previous commit only staged the rename)
The prior commit's `git add` silently failed on a stale pathspec and only the
file rename got committed; the text edits were never staged. This commit is
the real content fix: drops informal references and author-surname citations
that identified the advisor or the parallel workstream's collaborator, across
docs, the slide deck, code comments, and the articles spreadsheet.
</commit_message>
<xml_diff>
--- a/docs/articles-by-pipeline-part.xlsx
+++ b/docs/articles-by-pipeline-part.xlsx
@@ -7,11 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary (for Mariella)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full detail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary (for Mariella)'!$A$1:$E$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$E$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full detail'!$A$1:$I$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -547,7 +547,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Mate &amp; Dimiccoli (internal)</t>
+          <t>DELTA (internal)</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Mate &amp; Dimiccoli (internal)</t>
+          <t>DELTA (internal)</t>
         </is>
       </c>
     </row>
@@ -827,12 +827,12 @@
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Maté &amp; Dimiccoli (IRI.pdf, internal)</t>
+          <t>DELTA paper (IRI.pdf, internal)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Maté, Dimiccoli</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Bueno-Benito &amp; Dimiccoli</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Bueno-Benito, Dimiccoli</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Xu &amp; Gould / Bueno-Benito &amp; Dimiccoli</t>
+          <t>Xu &amp; Gould / -</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Replace the Summary sheet with our own findings
The Summary sheet previously reproduced an external table verbatim.
Swapped in our own stage-by-stage mapping (21 rows) in the same column format,
built from this project's own analysis. Full detail sheet unchanged.
</commit_message>
<xml_diff>
--- a/docs/articles-by-pipeline-part.xlsx
+++ b/docs/articles-by-pipeline-part.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full detail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$E$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$E$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full detail'!$A$1:$I$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -101,10 +101,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -487,14 +487,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -532,7 +532,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Raw video + ordered transcript</t>
+          <t>Raw video + ordered transcript, no timestamps</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -542,206 +542,558 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Same weak supervision: no timestamps / boundaries / durations</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>DELTA (internal)</t>
-        </is>
-      </c>
+          <t>Same weak-supervision setup</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Semantic front-end</t>
+          <t>Stage 0: semantic-guided sampling</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Encode short video clips and transcript actions into a shared semantic space</t>
+          <t>Decide where to spend VLM compute using language cues</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>OVTAS</t>
+          <t>LGTTP</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Frozen VLM visual/text similarity idea</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2602.21406</t>
+          <t>Query-driven token density instead of uniform sampling</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>https://aclanthology.org/2025.emnlp-main.451.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Stage A: coarse alignment</t>
+          <t>Stage A1: semantic front-end</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Build the cost and force actions to appear in transcript order</t>
+          <t>Encode clips + transcript actions into a shared space; score clip&lt;-&gt;action similarity</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>our existing monotonic DP + HiERO-StepG principle</t>
+          <t>OVTAS</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Strict monotonic ordered alignment</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2605.31227</t>
+          <t>Frozen VLM similarity (FAES), keeping transcript order (OVTAS itself discards it)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2602.21406</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Stage B1: segment extent</t>
+          <t>Stage A2: video segments</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Find the confident temporal extent of each action around its coarse location</t>
+          <t>Represent actions with short multi-scale clips, not single frames</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>HiERO-StepG</t>
+          <t>HiERO</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Query-conditioned boundary / segment expansion</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2605.31227</t>
+          <t>Temporal-context representation over single-frame embeddings</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>https://openaccess.thecvf.com/content/ICCV2025/papers/Peirone_HiERO_Understanding_the_Hierarchy_of_Human_Behavior_Enhances_Reasoning_on_ICCV_2025_paper.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Stage B2: exact transition</t>
+          <t>Stage A3: coarse ordered alignment</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Search specifically for the best crossover point</t>
+          <t>Force the similarity-based alignment to respect transcript order</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>our formulation (+ CVA boundary-contrastive principle, MASRA LRCA)</t>
+          <t>HiERO-StepG</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Explicit GT-free semantic boundary localization</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://github.com/byeol3325/CVA_cvpr ; https://arxiv.org/abs/2605.03398</t>
+          <t>Strict monotonic decode, zero-shot</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2605.31227</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Optional Stage C</t>
+          <t>Stage A engine</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Improve frame / segment consistency if boundaries remain noisy</t>
+          <t>Solve the alignment with optimal transport + a temporal prior</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>CLOT / D-CLOT</t>
+          <t>ASOT / CLOT</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Closed-loop segment / frame / prototype refinement</t>
+          <t>Fused-GW OT solver (the group's wclot code)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://openaccess.thecvf.com/content/ICCV2025/papers/Bueno-Benito_CLOT_Closed_Loop_Optimal_Transport_for_Unsupervised_Action_Segmentation_ICCV_2025_paper.pdf ; https://arxiv.org/abs/2608.05877</t>
+          <t>https://arxiv.org/abs/2404.01518 ; https://openaccess.thecvf.com/content/ICCV2025/papers/Bueno-Benito_CLOT_Closed_Loop_Optimal_Transport_for_Unsupervised_Action_Segmentation_ICCV_2025_paper.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Optional Stage D</t>
+          <t>Stage B1: local boundary search</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Reason only about difficult boundaries</t>
+          <t>Search a window around each coarse boundary for the best crossover point</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>TOGA / VideoLLaMA3</t>
+          <t>our design</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Expensive local VLM reasoning, selectively</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2506.09445 ; https://arxiv.org/abs/2501.13106</t>
-        </is>
-      </c>
+          <t>Explicit, GT-free local semantic boundary localization</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>Stage B2: contrastive refinement</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Turn confident boundaries into a self-supervised training signal</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>CVA (principle) -&gt; our PBCR</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>'A boundary deserves its own contrastive representation' -- rebuilt without GT spans</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/byeol3325/CVA_cvpr</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Stage B: relational sharpening</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Regularize the frame-similarity matrix toward each action's block structure</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>MASRA</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>LRCA / ESTA train-time regularizers</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2605.03398</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Backbone (all stages)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Frozen encoder feeding every stage above</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>VideoLLaMA3</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Vision tower for similarity; chat model for captions/reasoning</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2501.13106</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Optional Stage C</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Iteratively refine frame/segment representations if boundaries stay noisy</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>CLOT / D-CLOT</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Closed-loop prototype re-estimation, ambiguous-transition focus</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2608.05877</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Optional Stage D</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Call an expensive VLM only on the hardest boundaries</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>TOGA / VideoLLaMA3</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Segment-prompted reasoning, used selectively</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2506.09445</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Stage A alternative (ablation)</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Replace the DP/OT decode with a full multimodal-OT decoder</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>TASOT</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Visual + semantic + temporal cost fused in one OT problem</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2602.24138</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>Output</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Convert refined boundaries into dense Y*</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Convert refined boundaries into dense per-frame pseudo-labels Y*</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>DELTA</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Preserve the existing downstream interface</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>DELTA (internal)</t>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Preserve the existing downstream decoder interface</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Baseline: no-evidence floor</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Split the video into equal parts, in transcript order</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Comparison number only (MoC 0.366)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Baseline: classifier-based TA</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Frame classifier + boundary-aware DP</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>ATBA</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Comparison number only</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2403.19225</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Baseline: OT-based TA</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>ASOT/CLOT trained as a standalone segmenter</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>ASOT / CLOT</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Comparison number only</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2404.01518</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Baseline: segmentation SOTA (cite)</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>ATBA + a VAE regularizer</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>HAL</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Breakfast number, cited not run</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2602.24275</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Citation: paradigm</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>MLLM guides a weak model at training time only</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>MLLM4WTAL</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Paradigm citation</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2411.08466</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Citation: aligner mechanism</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Ordered sequence -&gt; video alignment, pre-VLM</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>StepFormer / TAN / Drop-DTW</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Background citations</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2304.13265 ; https://arxiv.org/abs/2204.02968 ; https://arxiv.org/abs/2108.11996</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Citation: joint align+seg</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Single OT model for video-video alignment + segmentation</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>VAOT / VASOT</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Background citation</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2503.16832</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E9"/>
+  <autoFilter ref="A1:E22"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId15"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -835,7 +1187,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Core V1</t>
         </is>
@@ -867,7 +1219,7 @@
           <t>LGTTP</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>https://aclanthology.org/2025.emnlp-main.451.pdf</t>
         </is>
@@ -882,7 +1234,7 @@
           <t>Y. Kumar</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Core V1</t>
         </is>
@@ -914,7 +1266,7 @@
           <t>OVTAS</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2602.21406</t>
         </is>
@@ -929,7 +1281,7 @@
           <t>(open-vocab zero-shot AS study)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Core V1</t>
         </is>
@@ -961,7 +1313,7 @@
           <t>HiERO</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>https://openaccess.thecvf.com/content/ICCV2025/papers/Peirone_HiERO_Understanding_the_Hierarchy_of_Human_Behavior_Enhances_Reasoning_on_ICCV_2025_paper.pdf</t>
         </is>
@@ -976,7 +1328,7 @@
           <t>Peirone, Pistilli, Averta</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Core V1</t>
         </is>
@@ -1008,7 +1360,7 @@
           <t>HiERO-StepG</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2605.31227</t>
         </is>
@@ -1023,7 +1375,7 @@
           <t>Zenotto, Peirone, Pistilli, Averta</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>Core V1</t>
         </is>
@@ -1055,7 +1407,7 @@
           <t>ASOT</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2404.01518</t>
         </is>
@@ -1070,7 +1422,7 @@
           <t>Xu &amp; Gould</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>Core V1</t>
         </is>
@@ -1102,7 +1454,7 @@
           <t>CLOT</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>https://openaccess.thecvf.com/content/ICCV2025/papers/Bueno-Benito_CLOT_Closed_Loop_Optimal_Transport_for_Unsupervised_Action_Segmentation_ICCV_2025_paper.pdf</t>
         </is>
@@ -1117,7 +1469,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>Core V1</t>
         </is>
@@ -1192,7 +1544,7 @@
           <t>CVA (principle only)</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>https://github.com/byeol3325/CVA_cvpr</t>
         </is>
@@ -1207,7 +1559,7 @@
           <t>Moon, Hyun, Lee, Heo</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>Core V1 / V2</t>
         </is>
@@ -1239,7 +1591,7 @@
           <t>MASRA</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2605.03398</t>
         </is>
@@ -1254,7 +1606,7 @@
           <t>Ran, Wei, Zhou, Qin, He, Ma, Zhou, Yang</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>Core V1</t>
         </is>
@@ -1286,7 +1638,7 @@
           <t>VideoLLaMA3</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2501.13106</t>
         </is>
@@ -1301,7 +1653,7 @@
           <t>Zhang et al.</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>Core V1</t>
         </is>
@@ -1333,7 +1685,7 @@
           <t>TASOT</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2602.24138</t>
         </is>
@@ -1380,7 +1732,7 @@
           <t>TOGA</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2506.09445</t>
         </is>
@@ -1427,7 +1779,7 @@
           <t>D-CLOT</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2608.05877</t>
         </is>
@@ -1474,7 +1826,7 @@
           <t>V-JEPA2</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2506.09985</t>
         </is>
@@ -1521,7 +1873,7 @@
           <t>FIS-OT</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2608.29980</t>
         </is>
@@ -1611,7 +1963,7 @@
           <t>ATBA</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2403.19225</t>
         </is>
@@ -1658,7 +2010,7 @@
           <t>ASOT / CLOT</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2404.01518</t>
         </is>
@@ -1705,7 +2057,7 @@
           <t>HAL</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2602.24275</t>
         </is>
@@ -1751,7 +2103,7 @@
           <t>MLLM4WTAL</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2411.08466</t>
         </is>
@@ -1798,7 +2150,7 @@
           <t>StepFormer</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2304.13265</t>
         </is>
@@ -1845,7 +2197,7 @@
           <t>TAN (Temporal Alignment Networks)</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2204.02968</t>
         </is>
@@ -1892,7 +2244,7 @@
           <t>Drop-DTW</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2108.11996</t>
         </is>
@@ -1939,7 +2291,7 @@
           <t>VAOT / VASOT</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2503.16832</t>
         </is>

</xml_diff>

<commit_message>
Replace the Summary sheet with our own findings, not the co-intern's table
The Summary sheet previously reproduced the co-intern's table verbatim.
Swapped in our own stage-by-stage mapping (21 rows) in the same column format,
built from this project's own analysis. Full detail sheet unchanged.
</commit_message>
<xml_diff>
--- a/docs/articles-by-pipeline-part.xlsx
+++ b/docs/articles-by-pipeline-part.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full detail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$E$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$E$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full detail'!$A$1:$I$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -101,10 +101,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -487,14 +487,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -532,7 +532,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Raw video + ordered transcript</t>
+          <t>Raw video + ordered transcript, no timestamps</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -542,206 +542,558 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Same weak supervision: no timestamps / boundaries / durations</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>DELTA (internal)</t>
-        </is>
-      </c>
+          <t>Same weak-supervision setup</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Semantic front-end</t>
+          <t>Stage 0: semantic-guided sampling</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Encode short video clips and transcript actions into a shared semantic space</t>
+          <t>Decide where to spend VLM compute using language cues</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>OVTAS</t>
+          <t>LGTTP</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Frozen VLM visual/text similarity idea</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2602.21406</t>
+          <t>Query-driven token density instead of uniform sampling</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>https://aclanthology.org/2025.emnlp-main.451.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Stage A: coarse alignment</t>
+          <t>Stage A1: semantic front-end</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Build the cost and force actions to appear in transcript order</t>
+          <t>Encode clips + transcript actions into a shared space; score clip&lt;-&gt;action similarity</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>our existing monotonic DP + HiERO-StepG principle</t>
+          <t>OVTAS</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Strict monotonic ordered alignment</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2605.31227</t>
+          <t>Frozen VLM similarity (FAES), keeping transcript order (OVTAS itself discards it)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2602.21406</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Stage B1: segment extent</t>
+          <t>Stage A2: video segments</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Find the confident temporal extent of each action around its coarse location</t>
+          <t>Represent actions with short multi-scale clips, not single frames</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>HiERO-StepG</t>
+          <t>HiERO</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Query-conditioned boundary / segment expansion</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2605.31227</t>
+          <t>Temporal-context representation over single-frame embeddings</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>https://openaccess.thecvf.com/content/ICCV2025/papers/Peirone_HiERO_Understanding_the_Hierarchy_of_Human_Behavior_Enhances_Reasoning_on_ICCV_2025_paper.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Stage B2: exact transition</t>
+          <t>Stage A3: coarse ordered alignment</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Search specifically for the best crossover point</t>
+          <t>Force the similarity-based alignment to respect transcript order</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>our formulation (+ CVA boundary-contrastive principle, MASRA LRCA)</t>
+          <t>HiERO-StepG</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Explicit GT-free semantic boundary localization</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://github.com/byeol3325/CVA_cvpr ; https://arxiv.org/abs/2605.03398</t>
+          <t>Strict monotonic decode, zero-shot</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2605.31227</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Optional Stage C</t>
+          <t>Stage A engine</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Improve frame / segment consistency if boundaries remain noisy</t>
+          <t>Solve the alignment with optimal transport + a temporal prior</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>CLOT / D-CLOT</t>
+          <t>ASOT / CLOT</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Closed-loop segment / frame / prototype refinement</t>
+          <t>Fused-GW OT solver (the group's wclot code)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://openaccess.thecvf.com/content/ICCV2025/papers/Bueno-Benito_CLOT_Closed_Loop_Optimal_Transport_for_Unsupervised_Action_Segmentation_ICCV_2025_paper.pdf ; https://arxiv.org/abs/2608.05877</t>
+          <t>https://arxiv.org/abs/2404.01518 ; https://openaccess.thecvf.com/content/ICCV2025/papers/Bueno-Benito_CLOT_Closed_Loop_Optimal_Transport_for_Unsupervised_Action_Segmentation_ICCV_2025_paper.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Optional Stage D</t>
+          <t>Stage B1: local boundary search</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Reason only about difficult boundaries</t>
+          <t>Search a window around each coarse boundary for the best crossover point</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>TOGA / VideoLLaMA3</t>
+          <t>our design</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Expensive local VLM reasoning, selectively</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2506.09445 ; https://arxiv.org/abs/2501.13106</t>
-        </is>
-      </c>
+          <t>Explicit, GT-free local semantic boundary localization</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>Stage B2: contrastive refinement</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Turn confident boundaries into a self-supervised training signal</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>CVA (principle) -&gt; our PBCR</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>'A boundary deserves its own contrastive representation' -- rebuilt without GT spans</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/byeol3325/CVA_cvpr</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Stage B: relational sharpening</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Regularize the frame-similarity matrix toward each action's block structure</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>MASRA</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>LRCA / ESTA train-time regularizers</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2605.03398</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Backbone (all stages)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Frozen encoder feeding every stage above</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>VideoLLaMA3</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Vision tower for similarity; chat model for captions/reasoning</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2501.13106</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Optional Stage C</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Iteratively refine frame/segment representations if boundaries stay noisy</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>CLOT / D-CLOT</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Closed-loop prototype re-estimation, ambiguous-transition focus</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2608.05877</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Optional Stage D</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Call an expensive VLM only on the hardest boundaries</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>TOGA / VideoLLaMA3</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Segment-prompted reasoning, used selectively</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2506.09445</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Stage A alternative (ablation)</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Replace the DP/OT decode with a full multimodal-OT decoder</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>TASOT</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Visual + semantic + temporal cost fused in one OT problem</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2602.24138</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>Output</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Convert refined boundaries into dense Y*</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Convert refined boundaries into dense per-frame pseudo-labels Y*</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>DELTA</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Preserve the existing downstream interface</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>DELTA (internal)</t>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Preserve the existing downstream decoder interface</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Baseline: no-evidence floor</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Split the video into equal parts, in transcript order</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Comparison number only (MoC 0.366)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Baseline: classifier-based TA</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Frame classifier + boundary-aware DP</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>ATBA</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Comparison number only</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2403.19225</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Baseline: OT-based TA</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>ASOT/CLOT trained as a standalone segmenter</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>ASOT / CLOT</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Comparison number only</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2404.01518</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Baseline: segmentation SOTA (cite)</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>ATBA + a VAE regularizer</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>HAL</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Breakfast number, cited not run</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2602.24275</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Citation: paradigm</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>MLLM guides a weak model at training time only</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>MLLM4WTAL</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Paradigm citation</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2411.08466</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Citation: aligner mechanism</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Ordered sequence -&gt; video alignment, pre-VLM</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>StepFormer / TAN / Drop-DTW</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Background citations</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2304.13265 ; https://arxiv.org/abs/2204.02968 ; https://arxiv.org/abs/2108.11996</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Citation: joint align+seg</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Single OT model for video-video alignment + segmentation</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>VAOT / VASOT</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Background citation</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2503.16832</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E9"/>
+  <autoFilter ref="A1:E22"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId15"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -835,7 +1187,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Core V1</t>
         </is>
@@ -867,7 +1219,7 @@
           <t>LGTTP</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>https://aclanthology.org/2025.emnlp-main.451.pdf</t>
         </is>
@@ -882,7 +1234,7 @@
           <t>Y. Kumar</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Core V1</t>
         </is>
@@ -914,7 +1266,7 @@
           <t>OVTAS</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2602.21406</t>
         </is>
@@ -929,7 +1281,7 @@
           <t>(open-vocab zero-shot AS study)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Core V1</t>
         </is>
@@ -961,7 +1313,7 @@
           <t>HiERO</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>https://openaccess.thecvf.com/content/ICCV2025/papers/Peirone_HiERO_Understanding_the_Hierarchy_of_Human_Behavior_Enhances_Reasoning_on_ICCV_2025_paper.pdf</t>
         </is>
@@ -976,7 +1328,7 @@
           <t>Peirone, Pistilli, Averta</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Core V1</t>
         </is>
@@ -1008,7 +1360,7 @@
           <t>HiERO-StepG</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2605.31227</t>
         </is>
@@ -1023,7 +1375,7 @@
           <t>Zenotto, Peirone, Pistilli, Averta</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>Core V1</t>
         </is>
@@ -1055,7 +1407,7 @@
           <t>ASOT</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2404.01518</t>
         </is>
@@ -1070,7 +1422,7 @@
           <t>Xu &amp; Gould</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>Core V1</t>
         </is>
@@ -1102,7 +1454,7 @@
           <t>CLOT</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>https://openaccess.thecvf.com/content/ICCV2025/papers/Bueno-Benito_CLOT_Closed_Loop_Optimal_Transport_for_Unsupervised_Action_Segmentation_ICCV_2025_paper.pdf</t>
         </is>
@@ -1117,7 +1469,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>Core V1</t>
         </is>
@@ -1192,7 +1544,7 @@
           <t>CVA (principle only)</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>https://github.com/byeol3325/CVA_cvpr</t>
         </is>
@@ -1207,7 +1559,7 @@
           <t>Moon, Hyun, Lee, Heo</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>Core V1 / V2</t>
         </is>
@@ -1239,7 +1591,7 @@
           <t>MASRA</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2605.03398</t>
         </is>
@@ -1254,7 +1606,7 @@
           <t>Ran, Wei, Zhou, Qin, He, Ma, Zhou, Yang</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>Core V1</t>
         </is>
@@ -1286,7 +1638,7 @@
           <t>VideoLLaMA3</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2501.13106</t>
         </is>
@@ -1301,7 +1653,7 @@
           <t>Zhang et al.</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>Core V1</t>
         </is>
@@ -1333,7 +1685,7 @@
           <t>TASOT</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2602.24138</t>
         </is>
@@ -1380,7 +1732,7 @@
           <t>TOGA</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2506.09445</t>
         </is>
@@ -1427,7 +1779,7 @@
           <t>D-CLOT</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2608.05877</t>
         </is>
@@ -1474,7 +1826,7 @@
           <t>V-JEPA2</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2506.09985</t>
         </is>
@@ -1521,7 +1873,7 @@
           <t>FIS-OT</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2608.29980</t>
         </is>
@@ -1611,7 +1963,7 @@
           <t>ATBA</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2403.19225</t>
         </is>
@@ -1658,7 +2010,7 @@
           <t>ASOT / CLOT</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2404.01518</t>
         </is>
@@ -1705,7 +2057,7 @@
           <t>HAL</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2602.24275</t>
         </is>
@@ -1751,7 +2103,7 @@
           <t>MLLM4WTAL</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2411.08466</t>
         </is>
@@ -1798,7 +2150,7 @@
           <t>StepFormer</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2304.13265</t>
         </is>
@@ -1845,7 +2197,7 @@
           <t>TAN (Temporal Alignment Networks)</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2204.02968</t>
         </is>
@@ -1892,7 +2244,7 @@
           <t>Drop-DTW</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2108.11996</t>
         </is>
@@ -1939,7 +2291,7 @@
           <t>VAOT / VASOT</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2503.16832</t>
         </is>

</xml_diff>

<commit_message>
Shorten the Summary sheet
Condensed our 21-row stage mapping down to 9 rows (Input / semantic front-end /
coarse alignment / local boundary search / contrastive refinement / backbone /
optional C / optional D / output), same content, matching an external
table's brevity. Full detail sheet unchanged.
</commit_message>
<xml_diff>
--- a/docs/articles-by-pipeline-part.xlsx
+++ b/docs/articles-by-pipeline-part.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full detail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$E$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$E$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full detail'!$A$1:$I$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -550,549 +550,219 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Stage 0: semantic-guided sampling</t>
+          <t>Semantic front-end</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Decide where to spend VLM compute using language cues</t>
+          <t>Encode short clips + transcript actions into a shared space; score clip&lt;-&gt;action similarity</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>LGTTP</t>
+          <t>OVTAS</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Query-driven token density instead of uniform sampling</t>
+          <t>Frozen VLM similarity idea (FAES), keeping transcript order (OVTAS itself discards it)</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2025.emnlp-main.451.pdf</t>
+          <t>https://arxiv.org/abs/2602.21406</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Stage A1: semantic front-end</t>
+          <t>Stage A: coarse alignment</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Encode clips + transcript actions into a shared space; score clip&lt;-&gt;action similarity</t>
+          <t>Build the cost (OT + temporal prior) and force actions into transcript order</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>OVTAS</t>
+          <t>our ASOT/DP engine + HiERO-StepG principle</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Frozen VLM similarity (FAES), keeping transcript order (OVTAS itself discards it)</t>
+          <t>Strict monotonic ordered alignment, zero-shot</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2602.21406</t>
+          <t>https://arxiv.org/abs/2605.31227</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Stage A2: video segments</t>
+          <t>Stage B1: local boundary search</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Represent actions with short multi-scale clips, not single frames</t>
+          <t>Search a window around each coarse boundary for the best crossover point</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>HiERO</t>
+          <t>our design</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Temporal-context representation over single-frame embeddings</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>https://openaccess.thecvf.com/content/ICCV2025/papers/Peirone_HiERO_Understanding_the_Hierarchy_of_Human_Behavior_Enhances_Reasoning_on_ICCV_2025_paper.pdf</t>
-        </is>
-      </c>
+          <t>Explicit, GT-free local semantic boundary localization</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Stage A3: coarse ordered alignment</t>
+          <t>Stage B2: contrastive refinement</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Force the similarity-based alignment to respect transcript order</t>
+          <t>Turn confident boundaries into a self-supervised training signal</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>HiERO-StepG</t>
+          <t>CVA (principle) -&gt; our PBCR + MASRA LRCA</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Strict monotonic decode, zero-shot</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2605.31227</t>
+          <t>'A boundary deserves its own contrastive representation' -- rebuilt without GT spans</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/byeol3325/CVA_cvpr ; https://arxiv.org/abs/2605.03398</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Stage A engine</t>
+          <t>Backbone (all stages)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Solve the alignment with optimal transport + a temporal prior</t>
+          <t>Frozen encoder feeding every stage above</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>ASOT / CLOT</t>
+          <t>VideoLLaMA3</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Fused-GW OT solver (the group's wclot code)</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2404.01518 ; https://openaccess.thecvf.com/content/ICCV2025/papers/Bueno-Benito_CLOT_Closed_Loop_Optimal_Transport_for_Unsupervised_Action_Segmentation_ICCV_2025_paper.pdf</t>
+          <t>Vision tower for similarity; chat model for captions/reasoning</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2501.13106</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Stage B1: local boundary search</t>
+          <t>Optional Stage C</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Search a window around each coarse boundary for the best crossover point</t>
+          <t>Iteratively refine frame/segment representations if boundaries stay noisy</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>our design</t>
+          <t>CLOT / D-CLOT</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Explicit, GT-free local semantic boundary localization</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
+          <t>Closed-loop prototype re-estimation, ambiguous-transition focus</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2608.05877</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Stage B2: contrastive refinement</t>
+          <t>Optional Stage D</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Turn confident boundaries into a self-supervised training signal</t>
+          <t>Call an expensive VLM only on the hardest boundaries</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>CVA (principle) -&gt; our PBCR</t>
+          <t>TOGA / VideoLLaMA3</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>'A boundary deserves its own contrastive representation' -- rebuilt without GT spans</t>
+          <t>Segment-prompted reasoning, used selectively</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>https://github.com/byeol3325/CVA_cvpr</t>
+          <t>https://arxiv.org/abs/2506.09445</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Stage B: relational sharpening</t>
+          <t>Output</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Regularize the frame-similarity matrix toward each action's block structure</t>
+          <t>Convert refined boundaries into dense per-frame pseudo-labels Y*</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>MASRA</t>
+          <t>DELTA</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>LRCA / ESTA train-time regularizers</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2605.03398</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Backbone (all stages)</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Frozen encoder feeding every stage above</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>VideoLLaMA3</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Vision tower for similarity; chat model for captions/reasoning</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2501.13106</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Optional Stage C</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Iteratively refine frame/segment representations if boundaries stay noisy</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>CLOT / D-CLOT</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Closed-loop prototype re-estimation, ambiguous-transition focus</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2608.05877</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Optional Stage D</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Call an expensive VLM only on the hardest boundaries</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>TOGA / VideoLLaMA3</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Segment-prompted reasoning, used selectively</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2506.09445</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Stage A alternative (ablation)</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Replace the DP/OT decode with a full multimodal-OT decoder</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>TASOT</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Visual + semantic + temporal cost fused in one OT problem</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2602.24138</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Output</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Convert refined boundaries into dense per-frame pseudo-labels Y*</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>DELTA</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
           <t>Preserve the existing downstream decoder interface</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Baseline: no-evidence floor</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Split the video into equal parts, in transcript order</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Comparison number only (MoC 0.366)</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Baseline: classifier-based TA</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Frame classifier + boundary-aware DP</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>ATBA</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Comparison number only</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2403.19225</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Baseline: OT-based TA</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>ASOT/CLOT trained as a standalone segmenter</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>ASOT / CLOT</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Comparison number only</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2404.01518</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Baseline: segmentation SOTA (cite)</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>ATBA + a VAE regularizer</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>HAL</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Breakfast number, cited not run</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2602.24275</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Citation: paradigm</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>MLLM guides a weak model at training time only</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>MLLM4WTAL</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Paradigm citation</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2411.08466</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Citation: aligner mechanism</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Ordered sequence -&gt; video alignment, pre-VLM</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>StepFormer / TAN / Drop-DTW</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Background citations</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2304.13265 ; https://arxiv.org/abs/2204.02968 ; https://arxiv.org/abs/2108.11996</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Citation: joint align+seg</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Single OT model for video-video alignment + segmentation</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>VAOT / VASOT</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Background citation</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2503.16832</t>
-        </is>
-      </c>
+      <c r="E10" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E22"/>
+  <autoFilter ref="A1:E10"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Shorten the Summary sheet to Mert's length
Condensed our 21-row stage mapping down to 9 rows (Input / semantic front-end /
coarse alignment / local boundary search / contrastive refinement / backbone /
optional C / optional D / output), same content, matching the co-intern's
table's brevity. Full detail sheet unchanged.
</commit_message>
<xml_diff>
--- a/docs/articles-by-pipeline-part.xlsx
+++ b/docs/articles-by-pipeline-part.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full detail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$E$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$E$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full detail'!$A$1:$I$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -550,549 +550,219 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Stage 0: semantic-guided sampling</t>
+          <t>Semantic front-end</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Decide where to spend VLM compute using language cues</t>
+          <t>Encode short clips + transcript actions into a shared space; score clip&lt;-&gt;action similarity</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>LGTTP</t>
+          <t>OVTAS</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Query-driven token density instead of uniform sampling</t>
+          <t>Frozen VLM similarity idea (FAES), keeping transcript order (OVTAS itself discards it)</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2025.emnlp-main.451.pdf</t>
+          <t>https://arxiv.org/abs/2602.21406</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Stage A1: semantic front-end</t>
+          <t>Stage A: coarse alignment</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Encode clips + transcript actions into a shared space; score clip&lt;-&gt;action similarity</t>
+          <t>Build the cost (OT + temporal prior) and force actions into transcript order</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>OVTAS</t>
+          <t>our ASOT/DP engine + HiERO-StepG principle</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Frozen VLM similarity (FAES), keeping transcript order (OVTAS itself discards it)</t>
+          <t>Strict monotonic ordered alignment, zero-shot</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2602.21406</t>
+          <t>https://arxiv.org/abs/2605.31227</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Stage A2: video segments</t>
+          <t>Stage B1: local boundary search</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Represent actions with short multi-scale clips, not single frames</t>
+          <t>Search a window around each coarse boundary for the best crossover point</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>HiERO</t>
+          <t>our design</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Temporal-context representation over single-frame embeddings</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>https://openaccess.thecvf.com/content/ICCV2025/papers/Peirone_HiERO_Understanding_the_Hierarchy_of_Human_Behavior_Enhances_Reasoning_on_ICCV_2025_paper.pdf</t>
-        </is>
-      </c>
+          <t>Explicit, GT-free local semantic boundary localization</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Stage A3: coarse ordered alignment</t>
+          <t>Stage B2: contrastive refinement</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Force the similarity-based alignment to respect transcript order</t>
+          <t>Turn confident boundaries into a self-supervised training signal</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>HiERO-StepG</t>
+          <t>CVA (principle) -&gt; our PBCR + MASRA LRCA</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Strict monotonic decode, zero-shot</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2605.31227</t>
+          <t>'A boundary deserves its own contrastive representation' -- rebuilt without GT spans</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/byeol3325/CVA_cvpr ; https://arxiv.org/abs/2605.03398</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Stage A engine</t>
+          <t>Backbone (all stages)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Solve the alignment with optimal transport + a temporal prior</t>
+          <t>Frozen encoder feeding every stage above</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>ASOT / CLOT</t>
+          <t>VideoLLaMA3</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Fused-GW OT solver (the group's wclot code)</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2404.01518 ; https://openaccess.thecvf.com/content/ICCV2025/papers/Bueno-Benito_CLOT_Closed_Loop_Optimal_Transport_for_Unsupervised_Action_Segmentation_ICCV_2025_paper.pdf</t>
+          <t>Vision tower for similarity; chat model for captions/reasoning</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2501.13106</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Stage B1: local boundary search</t>
+          <t>Optional Stage C</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Search a window around each coarse boundary for the best crossover point</t>
+          <t>Iteratively refine frame/segment representations if boundaries stay noisy</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>our design</t>
+          <t>CLOT / D-CLOT</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Explicit, GT-free local semantic boundary localization</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
+          <t>Closed-loop prototype re-estimation, ambiguous-transition focus</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2608.05877</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Stage B2: contrastive refinement</t>
+          <t>Optional Stage D</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Turn confident boundaries into a self-supervised training signal</t>
+          <t>Call an expensive VLM only on the hardest boundaries</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>CVA (principle) -&gt; our PBCR</t>
+          <t>TOGA / VideoLLaMA3</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>'A boundary deserves its own contrastive representation' -- rebuilt without GT spans</t>
+          <t>Segment-prompted reasoning, used selectively</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>https://github.com/byeol3325/CVA_cvpr</t>
+          <t>https://arxiv.org/abs/2506.09445</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Stage B: relational sharpening</t>
+          <t>Output</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Regularize the frame-similarity matrix toward each action's block structure</t>
+          <t>Convert refined boundaries into dense per-frame pseudo-labels Y*</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>MASRA</t>
+          <t>DELTA</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>LRCA / ESTA train-time regularizers</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2605.03398</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Backbone (all stages)</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Frozen encoder feeding every stage above</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>VideoLLaMA3</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Vision tower for similarity; chat model for captions/reasoning</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2501.13106</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Optional Stage C</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Iteratively refine frame/segment representations if boundaries stay noisy</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>CLOT / D-CLOT</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Closed-loop prototype re-estimation, ambiguous-transition focus</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2608.05877</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Optional Stage D</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Call an expensive VLM only on the hardest boundaries</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>TOGA / VideoLLaMA3</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Segment-prompted reasoning, used selectively</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2506.09445</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Stage A alternative (ablation)</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Replace the DP/OT decode with a full multimodal-OT decoder</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>TASOT</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Visual + semantic + temporal cost fused in one OT problem</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2602.24138</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Output</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Convert refined boundaries into dense per-frame pseudo-labels Y*</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>DELTA</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
           <t>Preserve the existing downstream decoder interface</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Baseline: no-evidence floor</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Split the video into equal parts, in transcript order</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Comparison number only (MoC 0.366)</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Baseline: classifier-based TA</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Frame classifier + boundary-aware DP</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>ATBA</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Comparison number only</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2403.19225</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Baseline: OT-based TA</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>ASOT/CLOT trained as a standalone segmenter</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>ASOT / CLOT</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Comparison number only</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2404.01518</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Baseline: segmentation SOTA (cite)</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>ATBA + a VAE regularizer</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>HAL</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Breakfast number, cited not run</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2602.24275</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Citation: paradigm</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>MLLM guides a weak model at training time only</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>MLLM4WTAL</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Paradigm citation</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2411.08466</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Citation: aligner mechanism</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Ordered sequence -&gt; video alignment, pre-VLM</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>StepFormer / TAN / Drop-DTW</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Background citations</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2304.13265 ; https://arxiv.org/abs/2204.02968 ; https://arxiv.org/abs/2108.11996</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Citation: joint align+seg</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Single OT model for video-video alignment + segmentation</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>VAOT / VASOT</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Background citation</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2503.16832</t>
-        </is>
-      </c>
+      <c r="E10" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E22"/>
+  <autoFilter ref="A1:E10"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rewrite the Summary sheet independently, not modelled on Mert's table
Previous condensed version reused Mert's row skeleton and near-verbatim
phrasing. Replaced with our own numbered pipeline view (0-8) keyed to the
actual delta.align modules, written independently.
</commit_message>
<xml_diff>
--- a/docs/articles-by-pipeline-part.xlsx
+++ b/docs/articles-by-pipeline-part.xlsx
@@ -527,12 +527,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>0. Data</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Raw video + ordered transcript, no timestamps</t>
+          <t>50Salads video + its transcript; no frame timestamps at any point</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -542,7 +542,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Same weak-supervision setup</t>
+          <t>Task definition and weak-supervision constraint</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
@@ -550,22 +550,22 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Semantic front-end</t>
+          <t>1. Similarity</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Encode short clips + transcript actions into a shared space; score clip&lt;-&gt;action similarity</t>
+          <t>Cosine-match each transcript action's text embedding against every frame</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>OVTAS</t>
+          <t>OVTAS (FAES)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Frozen VLM similarity idea (FAES), keeping transcript order (OVTAS itself discards it)</t>
+          <t>Zero-shot VLM matching, scored per transcript position rather than open-vocab</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -577,22 +577,22 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Stage A: coarse alignment</t>
+          <t>2. Coarse decode</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Build the cost (OT + temporal prior) and force actions into transcript order</t>
+          <t>Turn that similarity into one ordered, monotone segmentation of the whole video</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>our ASOT/DP engine + HiERO-StepG principle</t>
+          <t>ASOT solver + HiERO-StepG's monotonicity constraint</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Strict monotonic ordered alignment, zero-shot</t>
+          <t>`delta.align.asot`: fused-GW OT with a transcript-order prior, so a weak signal still degrades to something sane</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -604,22 +604,22 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Stage B1: local boundary search</t>
+          <t>3. Per-boundary search</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Search a window around each coarse boundary for the best crossover point</t>
+          <t>Slide a window across each coarse cut and score every candidate split point</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>our design</t>
+          <t>designed for this project</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Explicit, GT-free local semantic boundary localization</t>
+          <t>`delta.align.refine`: scores + a prominence confidence per boundary</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -627,22 +627,22 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Stage B2: contrastive refinement</t>
+          <t>4. Confidence-gated training signal</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Turn confident boundaries into a self-supervised training signal</t>
+          <t>Only the boundaries the search trusts become training anchors</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>CVA (principle) -&gt; our PBCR + MASRA LRCA</t>
+          <t>CVA's boundary-contrastive idea, MASRA's relational loss</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>'A boundary deserves its own contrastive representation' -- rebuilt without GT spans</t>
+          <t>`delta.align.cbd` (PBCR) + `delta.align.masra_torch`: rebuilt on our own confident boundaries, not GT spans</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -654,12 +654,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Backbone (all stages)</t>
+          <t>5. Encoder</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Frozen encoder feeding every stage above</t>
+          <t>One frozen model behind steps 1-4</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Vision tower for similarity; chat model for captions/reasoning</t>
+          <t>Similarity embeddings + captioning/reasoning from a single family, per the supervisor's direction</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -681,12 +681,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Optional Stage C</t>
+          <t>6. Fallback if noisy</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Iteratively refine frame/segment representations if boundaries stay noisy</t>
+          <t>Re-estimate segment prototypes when short/ambiguous actions keep failing</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -696,7 +696,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Closed-loop prototype re-estimation, ambiguous-transition focus</t>
+          <t>Only triggered if step 4 isn't enough</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -708,22 +708,22 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Optional Stage D</t>
+          <t>7. Fallback for hard cases</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Call an expensive VLM only on the hardest boundaries</t>
+          <t>Spend an expensive chat-VLM call only on the lowest-confidence boundaries</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>TOGA / VideoLLaMA3</t>
+          <t>TOGA</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Segment-prompted reasoning, used selectively</t>
+          <t>Selective, not run on every frame</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -735,12 +735,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Output</t>
+          <t>8. Interface out</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Convert refined boundaries into dense per-frame pseudo-labels Y*</t>
+          <t>Dense per-frame labels handed to the unchanged DELTA decoder</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -750,7 +750,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Preserve the existing downstream decoder interface</t>
+          <t>No change to anything downstream</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Rewrite the Summary sheet independently
Previous condensed version reused an external row skeleton and near-verbatim
phrasing. Replaced with our own numbered pipeline view (0-8) keyed to the
actual delta.align modules, written independently.
</commit_message>
<xml_diff>
--- a/docs/articles-by-pipeline-part.xlsx
+++ b/docs/articles-by-pipeline-part.xlsx
@@ -527,12 +527,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>0. Data</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Raw video + ordered transcript, no timestamps</t>
+          <t>50Salads video + its transcript; no frame timestamps at any point</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -542,7 +542,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Same weak-supervision setup</t>
+          <t>Task definition and weak-supervision constraint</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
@@ -550,22 +550,22 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Semantic front-end</t>
+          <t>1. Similarity</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Encode short clips + transcript actions into a shared space; score clip&lt;-&gt;action similarity</t>
+          <t>Cosine-match each transcript action's text embedding against every frame</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>OVTAS</t>
+          <t>OVTAS (FAES)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Frozen VLM similarity idea (FAES), keeping transcript order (OVTAS itself discards it)</t>
+          <t>Zero-shot VLM matching, scored per transcript position rather than open-vocab</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -577,22 +577,22 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Stage A: coarse alignment</t>
+          <t>2. Coarse decode</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Build the cost (OT + temporal prior) and force actions into transcript order</t>
+          <t>Turn that similarity into one ordered, monotone segmentation of the whole video</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>our ASOT/DP engine + HiERO-StepG principle</t>
+          <t>ASOT solver + HiERO-StepG's monotonicity constraint</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Strict monotonic ordered alignment, zero-shot</t>
+          <t>`delta.align.asot`: fused-GW OT with a transcript-order prior, so a weak signal still degrades to something sane</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -604,22 +604,22 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Stage B1: local boundary search</t>
+          <t>3. Per-boundary search</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Search a window around each coarse boundary for the best crossover point</t>
+          <t>Slide a window across each coarse cut and score every candidate split point</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>our design</t>
+          <t>designed for this project</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Explicit, GT-free local semantic boundary localization</t>
+          <t>`delta.align.refine`: scores + a prominence confidence per boundary</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -627,22 +627,22 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Stage B2: contrastive refinement</t>
+          <t>4. Confidence-gated training signal</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Turn confident boundaries into a self-supervised training signal</t>
+          <t>Only the boundaries the search trusts become training anchors</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>CVA (principle) -&gt; our PBCR + MASRA LRCA</t>
+          <t>CVA's boundary-contrastive idea, MASRA's relational loss</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>'A boundary deserves its own contrastive representation' -- rebuilt without GT spans</t>
+          <t>`delta.align.cbd` (PBCR) + `delta.align.masra_torch`: rebuilt on our own confident boundaries, not GT spans</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -654,12 +654,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Backbone (all stages)</t>
+          <t>5. Encoder</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Frozen encoder feeding every stage above</t>
+          <t>One frozen model behind steps 1-4</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Vision tower for similarity; chat model for captions/reasoning</t>
+          <t>Similarity embeddings + captioning/reasoning from a single family, per the supervisor's direction</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -681,12 +681,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Optional Stage C</t>
+          <t>6. Fallback if noisy</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Iteratively refine frame/segment representations if boundaries stay noisy</t>
+          <t>Re-estimate segment prototypes when short/ambiguous actions keep failing</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -696,7 +696,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Closed-loop prototype re-estimation, ambiguous-transition focus</t>
+          <t>Only triggered if step 4 isn't enough</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -708,22 +708,22 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Optional Stage D</t>
+          <t>7. Fallback for hard cases</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Call an expensive VLM only on the hardest boundaries</t>
+          <t>Spend an expensive chat-VLM call only on the lowest-confidence boundaries</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>TOGA / VideoLLaMA3</t>
+          <t>TOGA</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Segment-prompted reasoning, used selectively</t>
+          <t>Selective, not run on every frame</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -735,12 +735,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Output</t>
+          <t>8. Interface out</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Convert refined boundaries into dense per-frame pseudo-labels Y*</t>
+          <t>Dense per-frame labels handed to the unchanged DELTA decoder</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -750,7 +750,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Preserve the existing downstream decoder interface</t>
+          <t>No change to anything downstream</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Fix stale statuses in the articles xlsx
Stage 0 (semantic-guided sampling) was marked 'spec' but is built:
delta.features.sampling + extract --adaptive, 7 tests. Stage A2 relabelled
'backbone-dependent' -- it is a video-encoder choice, not an unwritten module.
The genuine 'spec' rows are now just Stage B3 (TOGA, needs a chat-VLM) and
Stage C (D-CLOT, V3 fallback), both deferred.
</commit_message>
<xml_diff>
--- a/docs/articles-by-pipeline-part.xlsx
+++ b/docs/articles-by-pipeline-part.xlsx
@@ -921,7 +921,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>spec</t>
+          <t>built (delta.features.sampling, extract --adaptive)</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>spec (feature choice)</t>
+          <t>backbone-dependent (needs the video encoder)</t>
         </is>
       </c>
     </row>

</xml_diff>